<commit_message>
chore(config): 关卡表与 Luban 导出同步
- Levels/L01..L30 六表（EnemyData/EnemyList/RoundData/SceneInfo/LevelRating/LevelMap）手工调参结果
- Assets/ConfigJson 重新导出，LevelRating 运行时哈希随之更新
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/Levels/L01/LevelRating.xlsx
+++ b/Luban/Config/Datas/Levels/L01/LevelRating.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -812,7 +812,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>771a35134b5be09511e87492fdaf3faef2b980093dc6ebb6cb5c72ef688de8b5</t>
+          <t>0135233bbe9cd3e5595063faf8ef222cfca1c0806565061d900f507fd56db4ce</t>
         </is>
       </c>
     </row>

</xml_diff>